<commit_message>
Update timeline, references, and report
</commit_message>
<xml_diff>
--- a/timeline.xlsx
+++ b/timeline.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lakeheaduca-my.sharepoint.com/personal/qzhao9_lakeheadu_ca/Documents/Courses/COMP5800/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\COMP9800\github\gradproj\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="215" documentId="8_{EC9B67B7-2FAD-470E-8B00-C8A13E57E1F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6732899A-04D8-4870-B394-5C0705131BAD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{721C8E63-582E-4B98-A58D-D8412DB7FED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="318" xr2:uid="{68D6A853-EF2B-430F-9008-F9D80DCEA0AF}"/>
   </bookViews>
@@ -126,10 +126,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Review related literature</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Experiments (Exploratory Analysis)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -159,6 +155,10 @@
   </si>
   <si>
     <t>experiment log, analysis of result</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Review related literature &amp; Updating draft paper</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -408,10 +408,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -732,18 +728,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D59A35F-780A-4ABD-8AE1-6067AF976B7E}">
   <dimension ref="A2:W15"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="54" customWidth="1"/>
-    <col min="2" max="15" width="9.21875" style="9" customWidth="1"/>
-    <col min="16" max="16" width="8.21875" hidden="1" customWidth="1"/>
-    <col min="17" max="19" width="8.77734375" hidden="1" customWidth="1"/>
+    <col min="2" max="15" width="9.25" style="9" customWidth="1"/>
+    <col min="16" max="16" width="8.25" hidden="1" customWidth="1"/>
+    <col min="17" max="19" width="8.75" hidden="1" customWidth="1"/>
     <col min="20" max="20" width="7.6640625" hidden="1" customWidth="1"/>
-    <col min="21" max="22" width="8.21875" hidden="1" customWidth="1"/>
-    <col min="23" max="23" width="57.77734375" style="3" customWidth="1"/>
+    <col min="21" max="22" width="8.25" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="57.75" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:23" ht="42" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" ht="44" x14ac:dyDescent="0.3">
       <c r="B2" s="6">
         <v>45903</v>
       </c>
@@ -808,7 +804,7 @@
         <v>46041</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" ht="37" x14ac:dyDescent="0.3">
       <c r="B3" s="7" t="s">
         <v>0</v>
       </c>
@@ -873,7 +869,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="31.2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" ht="31" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>25</v>
       </c>
@@ -899,12 +895,12 @@
       <c r="U4" s="4"/>
       <c r="V4" s="4"/>
       <c r="W4" s="10" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="5" spans="1:23" ht="17.399999999999999" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" ht="17.5" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -931,9 +927,9 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="17.399999999999999" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" ht="17.5" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -960,9 +956,9 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:23" ht="17.399999999999999" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" ht="17.5" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -986,12 +982,12 @@
       <c r="U7" s="4"/>
       <c r="V7" s="4"/>
       <c r="W7" s="12" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="8" spans="1:23" ht="17.399999999999999" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" ht="17.5" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -1015,12 +1011,12 @@
       <c r="U8" s="4"/>
       <c r="V8" s="4"/>
       <c r="W8" s="10" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="9" spans="1:23" ht="17.399999999999999" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" ht="17.5" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -1044,10 +1040,10 @@
       <c r="U9" s="4"/>
       <c r="V9" s="4"/>
       <c r="W9" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23" ht="17.399999999999999" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" ht="17.5" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>22</v>
       </c>
@@ -1076,10 +1072,10 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="16.8" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:23" ht="16.8" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:23" ht="16.8" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="1:23" ht="16.8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:23" ht="16.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="1:23" ht="16.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="14" spans="1:23" ht="16.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="15" spans="1:23" ht="16.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1089,12 +1085,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F0E8FC0-52D5-47D9-B127-4D7CD10C0786}">
   <dimension ref="A2:P10"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" ht="46.8" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="46.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="1">
         <v>46027</v>
       </c>
@@ -1138,7 +1134,7 @@
         <v>46118</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="49.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="49.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
         <v>0</v>
       </c>
@@ -1182,7 +1178,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -1200,7 +1196,7 @@
       <c r="O4" s="4"/>
       <c r="P4" s="4"/>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -1218,7 +1214,7 @@
       <c r="O5" s="4"/>
       <c r="P5" s="4"/>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -1236,7 +1232,7 @@
       <c r="O6" s="4"/>
       <c r="P6" s="4"/>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -1254,7 +1250,7 @@
       <c r="O7" s="4"/>
       <c r="P7" s="4"/>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -1272,7 +1268,7 @@
       <c r="O8" s="4"/>
       <c r="P8" s="4"/>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1290,7 +1286,7 @@
       <c r="O9" s="4"/>
       <c r="P9" s="4"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
@@ -1317,7 +1313,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80A02EA7-D1BC-45C4-B560-608AED901319}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>